<commit_message>
Added phase7 for Graffana web updates
</commit_message>
<xml_diff>
--- a/k8s_self_healing_project_steps.xlsx
+++ b/k8s_self_healing_project_steps.xlsx
@@ -8,21 +8,34 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\Desktop\batch16a\capstoneproj-kubernetes\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CEB7D21E-21C2-4179-811B-C1069D8F1CE2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5E153376-9341-46C6-8266-D271EAF6111A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" firstSheet="5" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Roadmap" sheetId="1" r:id="rId1"/>
-    <sheet name="Phase1" sheetId="2" r:id="rId2"/>
-    <sheet name="Phase2" sheetId="3" r:id="rId3"/>
-    <sheet name="Phase3" sheetId="4" r:id="rId4"/>
-    <sheet name="Phase4" sheetId="5" r:id="rId5"/>
-    <sheet name="Phase5" sheetId="6" r:id="rId6"/>
-    <sheet name="Phase6" sheetId="7" r:id="rId7"/>
-    <sheet name="Observations" sheetId="8" r:id="rId8"/>
+    <sheet name="Projectdetails" sheetId="10" r:id="rId1"/>
+    <sheet name="Roadmap" sheetId="1" r:id="rId2"/>
+    <sheet name="Phase1" sheetId="2" r:id="rId3"/>
+    <sheet name="Phase2" sheetId="3" r:id="rId4"/>
+    <sheet name="Phase3" sheetId="4" r:id="rId5"/>
+    <sheet name="Phase4" sheetId="5" r:id="rId6"/>
+    <sheet name="Phase5" sheetId="6" r:id="rId7"/>
+    <sheet name="Phase6" sheetId="7" r:id="rId8"/>
+    <sheet name="Observations" sheetId="8" r:id="rId9"/>
+    <sheet name="Phase7" sheetId="9" r:id="rId10"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
@@ -165,7 +178,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="167" uniqueCount="155">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="278" uniqueCount="199">
   <si>
     <t>Phase</t>
   </si>
@@ -186,9 +199,6 @@
   </si>
   <si>
     <t>Install Docker Desktop</t>
-  </si>
-  <si>
-    <t>Install the software engine that runs containers (isolated software packages) on your laptop.</t>
   </si>
   <si>
     <t>Go to https://www.docker.com/products/docker-desktop/ 
@@ -851,12 +861,305 @@
   <si>
     <t>Simultaneously, the custom Prometheus alert will trigger, sending a message directly to team's slack channel</t>
   </si>
+  <si>
+    <t>Detailed tasks</t>
+  </si>
+  <si>
+    <t>Web Dashboard UI Integration</t>
+  </si>
+  <si>
+    <t xml:space="preserve">
+Add Dashboard Handler inside main.go</t>
+  </si>
+  <si>
+    <t>https://github.com/peri-2005/k8s-self-healing-stack/tree/main/cmd/healer</t>
+  </si>
+  <si>
+    <t>Grafana Setup &amp; Metrics Panel Queries</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Setup Data Sources </t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Open Grafana and navigate to </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="8"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>Connections &gt; Data Sources</t>
+    </r>
+  </si>
+  <si>
+    <t>Click Save &amp; Test</t>
+  </si>
+  <si>
+    <t>Configure Real-Time Performance &amp; Custom App Metrics Panels</t>
+  </si>
+  <si>
+    <t>el Name</t>
+  </si>
+  <si>
+    <t>Visualization Type</t>
+  </si>
+  <si>
+    <t>Target Metrics / PromQL Query Expression</t>
+  </si>
+  <si>
+    <t>Description</t>
+  </si>
+  <si>
+    <t>Cluster CPU Utilization</t>
+  </si>
+  <si>
+    <t>Time Series Line Chart</t>
+  </si>
+  <si>
+    <t>sum(rate(node_cpu_seconds_total{mode!="idle"}[5m]))</t>
+  </si>
+  <si>
+    <t>Tracks compute load across all infrastructure nodes.</t>
+  </si>
+  <si>
+    <t>Cluster Memory Throughput</t>
+  </si>
+  <si>
+    <t>sum(node_memory_MemTotal_bytes - node_memory_MemAvailable_bytes)</t>
+  </si>
+  <si>
+    <t>Displays global memory footprints in bytes.</t>
+  </si>
+  <si>
+    <t>Network Throughput (Rx/Tx)</t>
+  </si>
+  <si>
+    <t>sum(rate(node_network_receive_bytes_total[5m]))</t>
+  </si>
+  <si>
+    <t>Monitors active live data packets received across interfaces.</t>
+  </si>
+  <si>
+    <t>Auto-Healing Executions</t>
+  </si>
+  <si>
+    <t>Bar Gauge / Stat Panel</t>
+  </si>
+  <si>
+    <t>sum(auto_healing_actions_total) by (action, status)</t>
+  </si>
+  <si>
+    <t>Verification and Verification Testing Pipeline</t>
+  </si>
+  <si>
+    <t>bash</t>
+  </si>
+  <si>
+    <t>curl -H "Content-Type: application/json" -d '[{"labels":{"alertname":"KubePodCrashLooping","severity":"critical","pod":"auth-api-xyz","namespace":"production"},"annotations":{"summary":"Manual Verification Trigger Test","description":"Validating live infrastructure routing downstream via standard endpoint configs"}}]' http://localhost:9093/api/v1/alerts</t>
+  </si>
+  <si>
+    <t>curl http://localhost:8080/metrics | grep auto_healing</t>
+  </si>
+  <si>
+    <r>
+      <t>1. Test Alertmanager Routing Execution:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> Run a terminal command loop to manually inject a failing structural metric payload test down Alertmanager’s routing API node directly:</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">   2. Scrape Custom Go Engine App Target Metrics:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> Ensure the app properly prints metrics values by fetching the active state locally:</t>
+    </r>
+  </si>
+  <si>
+    <t>To build Grafana dashboard panels, use the following visualization types and optimized expressions:</t>
+  </si>
+  <si>
+    <t>Visualizes custom metrics counters exposed from  Go application endpoint.</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Click </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="8"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>Add data source</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">, choose </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="8"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>Prometheus</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">, and specify server endpoint URL (e.g., </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="7"/>
+        <color theme="1"/>
+        <rFont val="Courier New"/>
+        <family val="3"/>
+      </rPr>
+      <t>http://cluster.local</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>).</t>
+    </r>
+  </si>
+  <si>
+    <t>Phase7</t>
+  </si>
+  <si>
+    <t>Tasks on a high level</t>
+  </si>
+  <si>
+    <t>Status</t>
+  </si>
+  <si>
+    <t>Done on 
+AWS 
+AND 
+Azure 
+cloud 
+platform</t>
+  </si>
+  <si>
+    <t>Yet to start in this week,
+ complete before 31stoctober</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="9"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>Projectname</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="9"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">  :  Kubernetes self healing project given on August 20th</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="9"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>Team</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="9"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> : Aparna, Vivek Pathak, Vilas Elavande, Sailaja</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="9"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>Start date by the team</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="9"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> : October 15th</t>
+    </r>
+  </si>
+  <si>
+    <t>Install the software engine that runs containers (isolated software packages) on  laptop.</t>
+  </si>
+  <si>
+    <t>Open  terminal/command prompt and run:
+docker --version
+(Should return something like: Docker version 27.x.x)</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="15" x14ac:knownFonts="1">
+  <fonts count="24" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -959,6 +1262,65 @@
       <name val="Calibri"/>
       <family val="2"/>
     </font>
+    <font>
+      <b/>
+      <sz val="8"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="8"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="8"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="7"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="7"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="6"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="9"/>
+      <color rgb="FFFF0000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -968,7 +1330,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="9">
+  <borders count="15">
     <border>
       <left/>
       <right/>
@@ -1072,12 +1434,76 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="36">
+  <cellXfs count="89">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -1120,9 +1546,6 @@
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
@@ -1135,12 +1558,6 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1167,6 +1584,164 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -1470,8 +2045,8 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:E21"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5B02CA5B-678A-4907-B1EB-41DCC7A611AD}">
+  <dimension ref="A1:E24"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="59.453125" bestFit="1" customWidth="1"/>
@@ -1482,360 +2057,258 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A1" s="21" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="21" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="21" t="s">
-        <v>2</v>
-      </c>
-      <c r="D1" s="21" t="s">
+      <c r="A1" s="20"/>
+      <c r="B1" s="20"/>
+      <c r="C1" s="20"/>
+      <c r="D1" s="20" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="21" t="s">
+      <c r="E1" s="20" t="s">
         <v>4</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A2" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="B2" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="C2" s="2" t="s">
+      <c r="B2" s="74"/>
+      <c r="C2" s="74"/>
+      <c r="D2" s="74"/>
+      <c r="E2" s="74"/>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="B3" s="74"/>
+      <c r="C3" s="74"/>
+      <c r="D3" s="74"/>
+      <c r="E3" s="74"/>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="B4" s="74"/>
+      <c r="C4" s="74"/>
+      <c r="D4" s="74"/>
+      <c r="E4" s="74"/>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A5" s="2"/>
+      <c r="B5" s="2"/>
+      <c r="C5" s="2"/>
+      <c r="D5" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="D2" s="2" t="s">
+      <c r="E5" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="E2" s="2" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A3" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="B3" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="C3" s="2" t="s">
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A6" s="2"/>
+      <c r="B6" s="2"/>
+      <c r="C6" s="2"/>
+      <c r="D6" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="D3" s="2" t="s">
+      <c r="E6" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="E3" s="2" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A4" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="B4" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="C4" s="2" t="s">
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A7" s="2"/>
+      <c r="B7" s="2"/>
+      <c r="C7" s="2"/>
+      <c r="D7" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="D4" s="2" t="s">
+      <c r="E7" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="E4" s="2" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A5" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="B5" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="C5" s="2" t="s">
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A8" s="2"/>
+      <c r="B8" s="2"/>
+      <c r="C8" s="2"/>
+      <c r="D8" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="D5" s="2" t="s">
+      <c r="E8" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="E5" s="2" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A6" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="B6" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="C6" s="2" t="s">
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A9" s="2"/>
+      <c r="B9" s="2"/>
+      <c r="C9" s="2"/>
+      <c r="D9" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="D6" s="2" t="s">
+      <c r="E9" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="E6" s="2" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A7" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="B7" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="C7" s="2" t="s">
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A10" s="74" t="s">
+        <v>194</v>
+      </c>
+      <c r="B10" s="2"/>
+      <c r="C10" s="2"/>
+      <c r="D10" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="D7" s="2" t="s">
+      <c r="E10" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="E7" s="2" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A8" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="B8" s="2" t="s">
-        <v>32</v>
-      </c>
-      <c r="C8" s="2" t="s">
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A11" s="74" t="s">
+        <v>195</v>
+      </c>
+      <c r="B11" s="2"/>
+      <c r="C11" s="2"/>
+      <c r="D11" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="D8" s="2" t="s">
+      <c r="E11" s="2" t="s">
         <v>34</v>
       </c>
-      <c r="E8" s="2" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A9" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="B9" s="2" t="s">
-        <v>36</v>
-      </c>
-      <c r="C9" s="2" t="s">
+    </row>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A12" s="74" t="s">
+        <v>196</v>
+      </c>
+      <c r="B12" s="2"/>
+      <c r="C12" s="2"/>
+      <c r="D12" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="D9" s="2" t="s">
+      <c r="E12" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="E9" s="2" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A10" s="2" t="s">
-        <v>40</v>
-      </c>
-      <c r="B10" s="2" t="s">
-        <v>41</v>
-      </c>
-      <c r="C10" s="2" t="s">
+    </row>
+    <row r="13" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A13" s="2"/>
+      <c r="B13" s="2"/>
+      <c r="C13" s="2"/>
+      <c r="D13" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="D10" s="2" t="s">
+      <c r="E13" s="2" t="s">
         <v>43</v>
       </c>
-      <c r="E10" s="2" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A11" s="2" t="s">
-        <v>40</v>
-      </c>
-      <c r="B11" s="2" t="s">
-        <v>45</v>
-      </c>
-      <c r="C11" s="2" t="s">
+    </row>
+    <row r="14" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A14" s="2"/>
+      <c r="B14" s="2"/>
+      <c r="C14" s="2"/>
+      <c r="D14" s="2" t="s">
         <v>46</v>
       </c>
-      <c r="D11" s="2" t="s">
+      <c r="E14" s="2" t="s">
         <v>47</v>
       </c>
-      <c r="E11" s="2" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A12" s="2" t="s">
-        <v>49</v>
-      </c>
-      <c r="B12" s="2" t="s">
-        <v>50</v>
-      </c>
-      <c r="C12" s="2" t="s">
+    </row>
+    <row r="15" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A15" s="2"/>
+      <c r="B15" s="2"/>
+      <c r="C15" s="2"/>
+      <c r="D15" s="2" t="s">
         <v>51</v>
       </c>
-      <c r="D12" s="2" t="s">
+      <c r="E15" s="2" t="s">
         <v>52</v>
       </c>
-      <c r="E12" s="2" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A13" s="2" t="s">
-        <v>49</v>
-      </c>
-      <c r="B13" s="2" t="s">
-        <v>54</v>
-      </c>
-      <c r="C13" s="2" t="s">
+    </row>
+    <row r="16" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A16" s="2"/>
+      <c r="B16" s="2"/>
+      <c r="C16" s="2"/>
+      <c r="D16" s="2" t="s">
         <v>55</v>
       </c>
-      <c r="D13" s="2" t="s">
+      <c r="E16" s="2" t="s">
         <v>56</v>
       </c>
-      <c r="E13" s="2" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A14" s="2" t="s">
-        <v>49</v>
-      </c>
-      <c r="B14" s="2" t="s">
-        <v>58</v>
-      </c>
-      <c r="C14" s="2" t="s">
+    </row>
+    <row r="17" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A17" s="2"/>
+      <c r="B17" s="2"/>
+      <c r="C17" s="2"/>
+      <c r="D17" s="2" t="s">
         <v>59</v>
       </c>
-      <c r="D14" s="2" t="s">
+      <c r="E17" s="2" t="s">
         <v>60</v>
       </c>
-      <c r="E14" s="2" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A15" s="2" t="s">
-        <v>62</v>
-      </c>
-      <c r="B15" s="2" t="s">
-        <v>63</v>
-      </c>
-      <c r="C15" s="2" t="s">
+    </row>
+    <row r="18" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A18" s="2"/>
+      <c r="B18" s="2"/>
+      <c r="C18" s="2"/>
+      <c r="D18" s="2" t="s">
         <v>64</v>
       </c>
-      <c r="D15" s="2" t="s">
+      <c r="E18" s="2" t="s">
         <v>65</v>
       </c>
-      <c r="E15" s="2" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A16" s="2" t="s">
-        <v>62</v>
-      </c>
-      <c r="B16" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="C16" s="2" t="s">
+    </row>
+    <row r="19" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A19" s="2"/>
+      <c r="B19" s="2"/>
+      <c r="C19" s="2"/>
+      <c r="D19" s="2" t="s">
         <v>68</v>
       </c>
-      <c r="D16" s="2" t="s">
+      <c r="E19" s="2" t="s">
         <v>69</v>
       </c>
-      <c r="E16" s="2" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A17" s="2" t="s">
-        <v>62</v>
-      </c>
-      <c r="B17" s="2" t="s">
-        <v>71</v>
-      </c>
-      <c r="C17" s="2" t="s">
+    </row>
+    <row r="20" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A20" s="2"/>
+      <c r="B20" s="2"/>
+      <c r="C20" s="2"/>
+      <c r="D20" s="2" t="s">
         <v>72</v>
       </c>
-      <c r="D17" s="2" t="s">
+      <c r="E20" s="2" t="s">
         <v>73</v>
       </c>
-      <c r="E17" s="2" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A18" s="2" t="s">
-        <v>75</v>
-      </c>
-      <c r="B18" s="2" t="s">
-        <v>76</v>
-      </c>
-      <c r="C18" s="2" t="s">
+    </row>
+    <row r="21" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A21" s="2"/>
+      <c r="B21" s="2"/>
+      <c r="C21" s="2"/>
+      <c r="D21" s="2" t="s">
         <v>77</v>
       </c>
-      <c r="D18" s="2" t="s">
+      <c r="E21" s="2" t="s">
         <v>78</v>
       </c>
-      <c r="E18" s="2" t="s">
-        <v>79</v>
-      </c>
-    </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A19" s="2" t="s">
-        <v>75</v>
-      </c>
-      <c r="B19" s="2" t="s">
-        <v>80</v>
-      </c>
-      <c r="C19" s="2" t="s">
+    </row>
+    <row r="22" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A22" s="2"/>
+      <c r="B22" s="2"/>
+      <c r="C22" s="2"/>
+      <c r="D22" s="2" t="s">
         <v>81</v>
       </c>
-      <c r="D19" s="2" t="s">
+      <c r="E22" s="2" t="s">
         <v>82</v>
       </c>
-      <c r="E19" s="2" t="s">
-        <v>83</v>
-      </c>
-    </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A20" s="2" t="s">
-        <v>84</v>
-      </c>
-      <c r="B20" s="2" t="s">
-        <v>85</v>
-      </c>
-      <c r="C20" s="2" t="s">
+    </row>
+    <row r="23" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A23" s="2"/>
+      <c r="B23" s="2"/>
+      <c r="C23" s="2"/>
+      <c r="D23" s="2" t="s">
         <v>86</v>
       </c>
-      <c r="D20" s="2" t="s">
+      <c r="E23" s="2" t="s">
         <v>87</v>
       </c>
-      <c r="E20" s="2" t="s">
-        <v>88</v>
-      </c>
-    </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A21" s="2" t="s">
-        <v>84</v>
-      </c>
-      <c r="B21" s="2" t="s">
-        <v>89</v>
-      </c>
-      <c r="C21" s="2" t="s">
+    </row>
+    <row r="24" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A24" s="2"/>
+      <c r="B24" s="2"/>
+      <c r="C24" s="2"/>
+      <c r="D24" s="2" t="s">
         <v>90</v>
       </c>
-      <c r="D21" s="2" t="s">
+      <c r="E24" s="2" t="s">
         <v>91</v>
-      </c>
-      <c r="E21" s="2" t="s">
-        <v>92</v>
       </c>
     </row>
   </sheetData>
@@ -1843,149 +2316,897 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{685DC4D0-D55A-4AD3-B758-6531B9A1AA33}">
+  <dimension ref="A2:I27"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="2" max="2" width="26.6328125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="86.26953125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="64.7265625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="20.1796875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="2" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A2" s="9"/>
+      <c r="B2" s="66" t="s">
+        <v>190</v>
+      </c>
+      <c r="C2" s="66"/>
+      <c r="D2" s="75" t="s">
+        <v>154</v>
+      </c>
+      <c r="E2" s="73"/>
+      <c r="I2" s="13" t="s">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A3" s="40" t="s">
+        <v>189</v>
+      </c>
+      <c r="B3" s="29" t="s">
+        <v>155</v>
+      </c>
+      <c r="C3" s="29"/>
+      <c r="D3" s="72" t="s">
+        <v>156</v>
+      </c>
+      <c r="E3" s="16" t="s">
+        <v>157</v>
+      </c>
+      <c r="I3" s="86" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A4" s="39"/>
+      <c r="B4" s="66" t="s">
+        <v>158</v>
+      </c>
+      <c r="C4" s="66"/>
+      <c r="D4" s="9" t="s">
+        <v>159</v>
+      </c>
+      <c r="E4" s="9"/>
+      <c r="I4" s="87"/>
+    </row>
+    <row r="5" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A5" s="39"/>
+      <c r="B5" s="24"/>
+      <c r="C5" s="24"/>
+      <c r="D5" s="9" t="s">
+        <v>160</v>
+      </c>
+      <c r="E5" s="9"/>
+      <c r="I5" s="87"/>
+    </row>
+    <row r="6" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A6" s="39"/>
+      <c r="B6" s="24"/>
+      <c r="C6" s="24"/>
+      <c r="D6" s="9" t="s">
+        <v>188</v>
+      </c>
+      <c r="E6" s="9"/>
+      <c r="I6" s="87"/>
+    </row>
+    <row r="7" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A7" s="39"/>
+      <c r="B7" s="24"/>
+      <c r="C7" s="24"/>
+      <c r="D7" s="9" t="s">
+        <v>161</v>
+      </c>
+      <c r="E7" s="9"/>
+      <c r="I7" s="87"/>
+    </row>
+    <row r="8" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A8" s="39"/>
+      <c r="B8" s="24"/>
+      <c r="C8" s="24"/>
+      <c r="D8" s="9" t="s">
+        <v>162</v>
+      </c>
+      <c r="E8" s="46" t="s">
+        <v>186</v>
+      </c>
+      <c r="I8" s="87"/>
+    </row>
+    <row r="9" spans="1:9" ht="45" x14ac:dyDescent="0.35">
+      <c r="A9" s="39"/>
+      <c r="B9" s="24"/>
+      <c r="C9" s="24"/>
+      <c r="D9" s="9"/>
+      <c r="E9" s="67" t="s">
+        <v>163</v>
+      </c>
+      <c r="F9" s="41" t="s">
+        <v>164</v>
+      </c>
+      <c r="G9" s="41" t="s">
+        <v>165</v>
+      </c>
+      <c r="H9" s="84" t="s">
+        <v>166</v>
+      </c>
+      <c r="I9" s="87"/>
+    </row>
+    <row r="10" spans="1:9" ht="47.5" x14ac:dyDescent="0.35">
+      <c r="A10" s="39"/>
+      <c r="B10" s="24"/>
+      <c r="C10" s="24"/>
+      <c r="D10" s="9"/>
+      <c r="E10" s="68" t="s">
+        <v>167</v>
+      </c>
+      <c r="F10" s="42" t="s">
+        <v>168</v>
+      </c>
+      <c r="G10" s="43" t="s">
+        <v>169</v>
+      </c>
+      <c r="H10" s="85" t="s">
+        <v>170</v>
+      </c>
+      <c r="I10" s="87"/>
+    </row>
+    <row r="11" spans="1:9" ht="57" x14ac:dyDescent="0.35">
+      <c r="A11" s="39"/>
+      <c r="B11" s="24"/>
+      <c r="C11" s="24"/>
+      <c r="D11" s="9"/>
+      <c r="E11" s="68" t="s">
+        <v>171</v>
+      </c>
+      <c r="F11" s="42" t="s">
+        <v>168</v>
+      </c>
+      <c r="G11" s="43" t="s">
+        <v>172</v>
+      </c>
+      <c r="H11" s="85" t="s">
+        <v>173</v>
+      </c>
+      <c r="I11" s="87"/>
+    </row>
+    <row r="12" spans="1:9" ht="54" x14ac:dyDescent="0.35">
+      <c r="A12" s="39"/>
+      <c r="B12" s="24"/>
+      <c r="C12" s="24"/>
+      <c r="D12" s="9"/>
+      <c r="E12" s="68" t="s">
+        <v>174</v>
+      </c>
+      <c r="F12" s="42" t="s">
+        <v>168</v>
+      </c>
+      <c r="G12" s="43" t="s">
+        <v>175</v>
+      </c>
+      <c r="H12" s="85" t="s">
+        <v>176</v>
+      </c>
+      <c r="I12" s="87"/>
+    </row>
+    <row r="13" spans="1:9" ht="72" x14ac:dyDescent="0.35">
+      <c r="A13" s="39"/>
+      <c r="B13" s="24"/>
+      <c r="C13" s="24"/>
+      <c r="D13" s="9"/>
+      <c r="E13" s="68" t="s">
+        <v>177</v>
+      </c>
+      <c r="F13" s="42" t="s">
+        <v>178</v>
+      </c>
+      <c r="G13" s="43" t="s">
+        <v>179</v>
+      </c>
+      <c r="H13" s="85" t="s">
+        <v>187</v>
+      </c>
+      <c r="I13" s="87"/>
+    </row>
+    <row r="14" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A14" s="39"/>
+      <c r="B14" s="24"/>
+      <c r="C14" s="24"/>
+      <c r="D14" s="9"/>
+    </row>
+    <row r="15" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A15" s="65"/>
+      <c r="B15" s="24"/>
+      <c r="C15" s="24"/>
+      <c r="D15" s="9"/>
+    </row>
+    <row r="16" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A16" s="9"/>
+      <c r="B16" s="9"/>
+      <c r="C16" s="9"/>
+      <c r="D16" s="9"/>
+    </row>
+    <row r="17" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A17" s="69" t="s">
+        <v>180</v>
+      </c>
+      <c r="B17" s="70"/>
+      <c r="C17" s="71"/>
+      <c r="D17" s="9"/>
+    </row>
+    <row r="18" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A18" s="44" t="s">
+        <v>184</v>
+      </c>
+      <c r="B18" s="9"/>
+      <c r="C18" s="9"/>
+      <c r="D18" s="9"/>
+    </row>
+    <row r="19" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A19" s="49" t="s">
+        <v>181</v>
+      </c>
+      <c r="B19" s="50"/>
+      <c r="C19" s="50"/>
+      <c r="D19" s="50"/>
+      <c r="E19" s="50"/>
+    </row>
+    <row r="20" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A20" s="45" t="s">
+        <v>182</v>
+      </c>
+      <c r="B20" s="9"/>
+      <c r="C20" s="9"/>
+      <c r="D20" s="9"/>
+    </row>
+    <row r="21" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A21" s="47"/>
+      <c r="B21" s="48"/>
+      <c r="C21" s="48"/>
+      <c r="D21" s="48"/>
+      <c r="E21" s="48"/>
+    </row>
+    <row r="22" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A22" s="51" t="s">
+        <v>185</v>
+      </c>
+      <c r="B22" s="52"/>
+      <c r="C22" s="52"/>
+      <c r="D22" s="53"/>
+    </row>
+    <row r="23" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A23" s="54" t="s">
+        <v>181</v>
+      </c>
+      <c r="B23" s="55"/>
+      <c r="C23" s="55"/>
+      <c r="D23" s="56"/>
+    </row>
+    <row r="24" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A24" s="57" t="s">
+        <v>183</v>
+      </c>
+      <c r="B24" s="58"/>
+      <c r="C24" s="58"/>
+      <c r="D24" s="59"/>
+    </row>
+    <row r="25" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A25" s="60"/>
+      <c r="B25" s="61"/>
+      <c r="C25" s="61"/>
+      <c r="D25" s="62"/>
+    </row>
+    <row r="26" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A26" s="63"/>
+      <c r="B26" s="64"/>
+      <c r="C26" s="64"/>
+      <c r="D26" s="64"/>
+      <c r="E26" s="64"/>
+    </row>
+    <row r="27" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A27" s="63"/>
+      <c r="B27" s="64"/>
+      <c r="C27" s="64"/>
+      <c r="D27" s="64"/>
+      <c r="E27" s="64"/>
+    </row>
+  </sheetData>
+  <mergeCells count="14">
+    <mergeCell ref="A26:E27"/>
+    <mergeCell ref="A3:A15"/>
+    <mergeCell ref="B5:C15"/>
+    <mergeCell ref="A17:C17"/>
+    <mergeCell ref="I3:I13"/>
+    <mergeCell ref="A21:E21"/>
+    <mergeCell ref="A19:E19"/>
+    <mergeCell ref="A22:D22"/>
+    <mergeCell ref="A23:D23"/>
+    <mergeCell ref="A24:D24"/>
+    <mergeCell ref="A25:D25"/>
+    <mergeCell ref="B2:C2"/>
+    <mergeCell ref="B3:C3"/>
+    <mergeCell ref="B4:C4"/>
+  </mergeCells>
+  <hyperlinks>
+    <hyperlink ref="E3" r:id="rId1" xr:uid="{90BA0A35-8D71-41A7-9D24-EF0B7981C4EE}"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId2"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:E24"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="59.453125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="42" customWidth="1"/>
+    <col min="3" max="3" width="107.453125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="255.6328125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="45" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A1" s="20" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="20" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="20" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="20" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="20" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A2" s="74"/>
+      <c r="B2" s="74"/>
+      <c r="C2" s="74"/>
+      <c r="D2" s="74"/>
+      <c r="E2" s="74"/>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A3" s="74"/>
+      <c r="B3" s="74"/>
+      <c r="C3" s="74"/>
+      <c r="D3" s="74"/>
+      <c r="E3" s="74"/>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A4" s="74"/>
+      <c r="B4" s="74"/>
+      <c r="C4" s="74"/>
+      <c r="D4" s="74"/>
+      <c r="E4" s="74"/>
+    </row>
+    <row r="5" spans="1:5" ht="36.5" x14ac:dyDescent="0.35">
+      <c r="A5" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="C5" s="2" t="s">
+        <v>197</v>
+      </c>
+      <c r="D5" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="E5" s="88" t="s">
+        <v>198</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A6" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="D6" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="E6" s="2" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A7" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="B7" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="C7" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="D7" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="E7" s="2" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A8" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="B8" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="C8" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="D8" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="E8" s="2" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A9" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="B9" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="C9" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="D9" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="E9" s="2" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A10" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="B10" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="C10" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="D10" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="E10" s="2" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A11" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="B11" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="C11" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="D11" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="E11" s="2" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A12" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="B12" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="C12" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="D12" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="E12" s="2" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A13" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="B13" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="C13" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="D13" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="E13" s="2" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A14" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="B14" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="C14" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="D14" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="E14" s="2" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A15" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="B15" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="C15" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="D15" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="E15" s="2" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A16" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="B16" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="C16" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="D16" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="E16" s="2" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A17" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="B17" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="C17" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="D17" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="E17" s="2" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A18" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="B18" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="C18" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="D18" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="E18" s="2" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A19" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="B19" s="2" t="s">
+        <v>66</v>
+      </c>
+      <c r="C19" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="D19" s="2" t="s">
+        <v>68</v>
+      </c>
+      <c r="E19" s="2" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A20" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="B20" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="C20" s="2" t="s">
+        <v>71</v>
+      </c>
+      <c r="D20" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="E20" s="2" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="21" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A21" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="B21" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="C21" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="D21" s="2" t="s">
+        <v>77</v>
+      </c>
+      <c r="E21" s="2" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="22" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A22" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="B22" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="C22" s="2" t="s">
+        <v>80</v>
+      </c>
+      <c r="D22" s="2" t="s">
+        <v>81</v>
+      </c>
+      <c r="E22" s="2" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="23" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A23" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="B23" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="C23" s="2" t="s">
+        <v>85</v>
+      </c>
+      <c r="D23" s="2" t="s">
+        <v>86</v>
+      </c>
+      <c r="E23" s="2" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="24" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A24" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="B24" s="2" t="s">
+        <v>88</v>
+      </c>
+      <c r="C24" s="2" t="s">
+        <v>89</v>
+      </c>
+      <c r="D24" s="2" t="s">
+        <v>90</v>
+      </c>
+      <c r="E24" s="2" t="s">
+        <v>91</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{68CAA0CE-0BB2-405D-8BBA-C50071D906C9}">
-  <dimension ref="A4:E21"/>
+  <dimension ref="A3:E21"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="2" max="2" width="51.81640625" customWidth="1"/>
     <col min="3" max="3" width="64.81640625" customWidth="1"/>
+    <col min="4" max="4" width="12.1796875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="4" spans="1:3" ht="36.5" x14ac:dyDescent="0.35">
-      <c r="A4" s="27" t="s">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A3" s="9"/>
+      <c r="B3" s="34" t="s">
+        <v>190</v>
+      </c>
+      <c r="C3" s="34" t="s">
+        <v>154</v>
+      </c>
+      <c r="D3" s="34" t="s">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" ht="36.5" x14ac:dyDescent="0.35">
+      <c r="A4" s="24" t="s">
+        <v>96</v>
+      </c>
+      <c r="B4" s="21" t="s">
+        <v>95</v>
+      </c>
+      <c r="C4" s="6" t="s">
+        <v>92</v>
+      </c>
+      <c r="D4" s="76" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A5" s="24"/>
+      <c r="B5" s="22"/>
+      <c r="C5" s="5" t="s">
+        <v>93</v>
+      </c>
+      <c r="D5" s="30"/>
+    </row>
+    <row r="6" spans="1:4" ht="58" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A6" s="24"/>
+      <c r="B6" s="22"/>
+      <c r="C6" s="5" t="s">
+        <v>94</v>
+      </c>
+      <c r="D6" s="30"/>
+    </row>
+    <row r="7" spans="1:4" ht="24.5" x14ac:dyDescent="0.35">
+      <c r="A7" s="24"/>
+      <c r="B7" s="23"/>
+      <c r="C7" s="5" t="s">
         <v>97</v>
       </c>
-      <c r="B4" s="22" t="s">
-        <v>96</v>
-      </c>
-      <c r="C4" s="6" t="s">
-        <v>93</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A5" s="27"/>
-      <c r="B5" s="23"/>
-      <c r="C5" s="5" t="s">
-        <v>94</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" ht="58" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A6" s="27"/>
-      <c r="B6" s="23"/>
-      <c r="C6" s="5" t="s">
-        <v>95</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3" ht="24.5" x14ac:dyDescent="0.35">
-      <c r="A7" s="27"/>
-      <c r="B7" s="24"/>
-      <c r="C7" s="5" t="s">
+      <c r="D7" s="30"/>
+    </row>
+    <row r="8" spans="1:4" ht="228.5" x14ac:dyDescent="0.35">
+      <c r="A8" s="24"/>
+      <c r="B8" s="77" t="s">
         <v>98</v>
       </c>
-    </row>
-    <row r="8" spans="1:3" ht="228.5" x14ac:dyDescent="0.35">
-      <c r="A8" s="27"/>
-      <c r="B8" s="20" t="s">
+      <c r="C8" s="4" t="s">
         <v>99</v>
       </c>
-      <c r="C8" s="4" t="s">
+      <c r="D8" s="30"/>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A9" s="24"/>
+      <c r="B9" s="78" t="s">
         <v>100</v>
       </c>
-    </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A9" s="27"/>
-      <c r="B9" s="25" t="s">
+      <c r="C9" s="3"/>
+      <c r="D9" s="30"/>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A10" s="24"/>
+      <c r="B10" s="78"/>
+      <c r="C10" s="7" t="s">
         <v>101</v>
       </c>
-      <c r="C9" s="3"/>
-    </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A10" s="27"/>
-      <c r="B10" s="26"/>
-      <c r="C10" s="7" t="s">
+      <c r="D10" s="30"/>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A11" s="24"/>
+      <c r="B11" s="78"/>
+      <c r="C11" s="7"/>
+      <c r="D11" s="30"/>
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A12" s="24"/>
+      <c r="B12" s="78"/>
+      <c r="C12" s="7" t="s">
         <v>102</v>
       </c>
-    </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A11" s="27"/>
-      <c r="B11" s="26"/>
-      <c r="C11" s="7"/>
-    </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A12" s="27"/>
-      <c r="B12" s="26"/>
-      <c r="C12" s="7" t="s">
+      <c r="D12" s="30"/>
+    </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A13" s="24"/>
+      <c r="B13" s="78"/>
+      <c r="C13" s="7" t="s">
         <v>103</v>
       </c>
-    </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A13" s="27"/>
-      <c r="B13" s="26"/>
-      <c r="C13" s="7" t="s">
+      <c r="D13" s="30"/>
+    </row>
+    <row r="14" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A14" s="24"/>
+      <c r="B14" s="78"/>
+      <c r="C14" s="7" t="s">
         <v>104</v>
       </c>
-    </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A14" s="27"/>
-      <c r="B14" s="26"/>
-      <c r="C14" s="7" t="s">
+      <c r="D14" s="30"/>
+    </row>
+    <row r="15" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A15" s="24"/>
+      <c r="B15" s="78"/>
+      <c r="C15" s="7" t="s">
         <v>105</v>
       </c>
-    </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A15" s="27"/>
-      <c r="B15" s="26"/>
-      <c r="C15" s="7" t="s">
+      <c r="D15" s="30"/>
+    </row>
+    <row r="16" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A16" s="24"/>
+      <c r="B16" s="78"/>
+      <c r="C16" s="7" t="s">
         <v>106</v>
       </c>
-    </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A16" s="27"/>
-      <c r="B16" s="26"/>
-      <c r="C16" s="7" t="s">
+      <c r="D16" s="30"/>
+    </row>
+    <row r="17" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A17" s="24"/>
+      <c r="B17" s="78"/>
+      <c r="C17" s="7" t="s">
         <v>107</v>
       </c>
-    </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A17" s="27"/>
-      <c r="B17" s="26"/>
-      <c r="C17" s="7" t="s">
+      <c r="D17" s="30"/>
+    </row>
+    <row r="18" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A18" s="24"/>
+      <c r="B18" s="78"/>
+      <c r="C18" s="7"/>
+      <c r="D18" s="30"/>
+    </row>
+    <row r="19" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A19" s="24"/>
+      <c r="B19" s="78"/>
+      <c r="C19" s="7" t="s">
         <v>108</v>
       </c>
-    </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A18" s="27"/>
-      <c r="B18" s="26"/>
-      <c r="C18" s="7"/>
-    </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A19" s="27"/>
-      <c r="B19" s="26"/>
-      <c r="C19" s="7" t="s">
+      <c r="D19" s="30"/>
+    </row>
+    <row r="20" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A20" s="24"/>
+      <c r="B20" s="78"/>
+      <c r="C20" s="7" t="s">
         <v>109</v>
       </c>
-    </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A20" s="27"/>
-      <c r="B20" s="26"/>
-      <c r="C20" s="7" t="s">
+      <c r="D20" s="30"/>
+    </row>
+    <row r="21" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A21" s="24"/>
+      <c r="B21" s="78"/>
+      <c r="C21" s="8" t="s">
         <v>110</v>
       </c>
-    </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A21" s="27"/>
-      <c r="B21" s="26"/>
-      <c r="C21" s="8" t="s">
-        <v>111</v>
-      </c>
+      <c r="D21" s="30"/>
       <c r="E21" s="2"/>
     </row>
   </sheetData>
-  <mergeCells count="3">
+  <mergeCells count="4">
     <mergeCell ref="B4:B7"/>
     <mergeCell ref="B9:B21"/>
     <mergeCell ref="A4:A21"/>
+    <mergeCell ref="D4:D21"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="C4" r:id="rId1" display="https://aws.amazon.com/" xr:uid="{36DFC495-525A-46D1-9D73-4DEDBA9C8C2F}"/>
@@ -1995,54 +3216,71 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E2B76E60-70CA-4F2B-ACC6-5BDEB6B512AD}">
-  <dimension ref="A3:C5"/>
+  <dimension ref="A2:D5"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="2" max="2" width="43.08984375" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="104.1796875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="3" spans="1:3" ht="174" x14ac:dyDescent="0.35">
-      <c r="A3" s="30" t="s">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="B2" s="34" t="s">
+        <v>190</v>
+      </c>
+      <c r="C2" s="34" t="s">
+        <v>154</v>
+      </c>
+      <c r="D2" t="s">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" ht="174" x14ac:dyDescent="0.35">
+      <c r="A3" s="27" t="s">
+        <v>113</v>
+      </c>
+      <c r="B3" s="11" t="s">
+        <v>111</v>
+      </c>
+      <c r="C3" s="1" t="s">
+        <v>112</v>
+      </c>
+      <c r="D3" s="79" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" ht="116" x14ac:dyDescent="0.35">
+      <c r="A4" s="28"/>
+      <c r="B4" s="25" t="s">
         <v>114</v>
       </c>
-      <c r="B3" s="11" t="s">
-        <v>112</v>
-      </c>
-      <c r="C3" s="1" t="s">
-        <v>113</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" ht="116" x14ac:dyDescent="0.35">
-      <c r="A4" s="31"/>
-      <c r="B4" s="28" t="s">
+      <c r="C4" s="12" t="s">
+        <v>116</v>
+      </c>
+      <c r="D4" s="79"/>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A5" s="29"/>
+      <c r="B5" s="26"/>
+      <c r="C5" s="10" t="s">
         <v>115</v>
       </c>
-      <c r="C4" s="12" t="s">
-        <v>117</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A5" s="32"/>
-      <c r="B5" s="29"/>
-      <c r="C5" s="10" t="s">
-        <v>116</v>
-      </c>
+      <c r="D5" s="79"/>
     </row>
   </sheetData>
-  <mergeCells count="2">
+  <mergeCells count="3">
     <mergeCell ref="B4:B5"/>
     <mergeCell ref="A3:A5"/>
+    <mergeCell ref="D3:D5"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{447C61BA-E553-4864-8B98-4F812738AF8C}">
-  <dimension ref="A3:D6"/>
+  <dimension ref="A2:E6"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="2" max="2" width="29.453125" bestFit="1" customWidth="1"/>
@@ -2050,54 +3288,74 @@
     <col min="4" max="4" width="43.6328125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="3" spans="1:4" ht="58" x14ac:dyDescent="0.35">
-      <c r="A3" s="30" t="s">
-        <v>127</v>
-      </c>
-      <c r="B3" s="30" t="s">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="B2" s="36" t="s">
+        <v>190</v>
+      </c>
+      <c r="C2" s="37"/>
+      <c r="D2" s="34" t="s">
+        <v>154</v>
+      </c>
+      <c r="E2" s="33" t="s">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" ht="87" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A3" s="27" t="s">
+        <v>126</v>
+      </c>
+      <c r="B3" s="27" t="s">
+        <v>117</v>
+      </c>
+      <c r="C3" s="13" t="s">
         <v>118</v>
       </c>
-      <c r="C3" s="13" t="s">
+      <c r="D3" s="12" t="s">
         <v>119</v>
       </c>
-      <c r="D3" s="12" t="s">
+      <c r="E3" s="76" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A4" s="28"/>
+      <c r="B4" s="28"/>
+      <c r="C4" s="14" t="s">
         <v>120</v>
       </c>
-    </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A4" s="31"/>
-      <c r="B4" s="31"/>
-      <c r="C4" s="14" t="s">
+      <c r="D4" s="16" t="s">
         <v>121</v>
       </c>
-      <c r="D4" s="16" t="s">
+      <c r="E4" s="76"/>
+    </row>
+    <row r="5" spans="1:5" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="A5" s="28"/>
+      <c r="B5" s="28"/>
+      <c r="C5" s="15" t="s">
         <v>122</v>
       </c>
-    </row>
-    <row r="5" spans="1:4" ht="43.5" x14ac:dyDescent="0.35">
-      <c r="A5" s="31"/>
-      <c r="B5" s="31"/>
-      <c r="C5" s="15" t="s">
+      <c r="D5" s="16" t="s">
         <v>123</v>
       </c>
-      <c r="D5" s="16" t="s">
+      <c r="E5" s="76"/>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A6" s="29"/>
+      <c r="B6" s="29"/>
+      <c r="C6" s="13" t="s">
         <v>124</v>
       </c>
-    </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A6" s="32"/>
-      <c r="B6" s="32"/>
-      <c r="C6" s="13" t="s">
+      <c r="D6" s="9" t="s">
         <v>125</v>
       </c>
-      <c r="D6" s="9" t="s">
-        <v>126</v>
-      </c>
+      <c r="E6" s="76"/>
     </row>
   </sheetData>
-  <mergeCells count="2">
+  <mergeCells count="4">
     <mergeCell ref="B3:B6"/>
     <mergeCell ref="A3:A6"/>
+    <mergeCell ref="B2:C2"/>
+    <mergeCell ref="E3:E6"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="D4" r:id="rId1" xr:uid="{8DBD36F9-D772-4FB6-BE46-095EFDA26637}"/>
@@ -2108,9 +3366,9 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{599BB6F7-480A-4659-98BB-552FC8F9F032}">
-  <dimension ref="A3:D4"/>
+  <dimension ref="A2:E4"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="2" max="2" width="40.54296875" bestFit="1" customWidth="1"/>
@@ -2118,34 +3376,52 @@
     <col min="4" max="4" width="49.1796875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="3" spans="1:4" ht="29" x14ac:dyDescent="0.35">
-      <c r="A3" s="33" t="s">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="B2" s="38" t="s">
+        <v>190</v>
+      </c>
+      <c r="C2" s="37"/>
+      <c r="D2" s="34" t="s">
+        <v>154</v>
+      </c>
+      <c r="E2" s="33" t="s">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" ht="29" x14ac:dyDescent="0.35">
+      <c r="A3" s="30" t="s">
+        <v>127</v>
+      </c>
+      <c r="B3" s="30" t="s">
         <v>128</v>
       </c>
-      <c r="B3" s="33" t="s">
+      <c r="C3" s="12" t="s">
         <v>129</v>
       </c>
-      <c r="C3" s="12" t="s">
+      <c r="D3" s="16" t="s">
         <v>130</v>
       </c>
-      <c r="D3" s="16" t="s">
+      <c r="E3" s="80" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" ht="58" x14ac:dyDescent="0.35">
+      <c r="A4" s="30"/>
+      <c r="B4" s="30"/>
+      <c r="C4" s="12" t="s">
         <v>131</v>
       </c>
-    </row>
-    <row r="4" spans="1:4" ht="58" x14ac:dyDescent="0.35">
-      <c r="A4" s="33"/>
-      <c r="B4" s="33"/>
-      <c r="C4" s="12" t="s">
+      <c r="D4" s="12" t="s">
         <v>132</v>
       </c>
-      <c r="D4" s="12" t="s">
-        <v>133</v>
-      </c>
+      <c r="E4" s="81"/>
     </row>
   </sheetData>
-  <mergeCells count="2">
+  <mergeCells count="4">
     <mergeCell ref="A3:A4"/>
     <mergeCell ref="B3:B4"/>
+    <mergeCell ref="B2:C2"/>
+    <mergeCell ref="E3:E4"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="D3" r:id="rId1" xr:uid="{4D04E255-2381-4B8B-95FB-EA09A0D6C5E1}"/>
@@ -2155,9 +3431,9 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{38606AF9-C385-4019-BEA1-3DA49CE31EDC}">
-  <dimension ref="A3:D6"/>
+  <dimension ref="A2:E6"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="2" max="2" width="44.1796875" bestFit="1" customWidth="1"/>
@@ -2165,57 +3441,77 @@
     <col min="4" max="4" width="109.7265625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A3" s="33" t="s">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="B2" s="38" t="s">
+        <v>190</v>
+      </c>
+      <c r="C2" s="37"/>
+      <c r="D2" s="34" t="s">
+        <v>154</v>
+      </c>
+      <c r="E2" s="9" t="s">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A3" s="30" t="s">
+        <v>133</v>
+      </c>
+      <c r="B3" s="31" t="s">
         <v>134</v>
       </c>
-      <c r="B3" s="34" t="s">
+      <c r="C3" s="14" t="s">
         <v>135</v>
       </c>
-      <c r="C3" s="14" t="s">
+      <c r="D3" s="16" t="s">
         <v>136</v>
       </c>
-      <c r="D3" s="16" t="s">
+      <c r="E3" s="82" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A4" s="30"/>
+      <c r="B4" s="31"/>
+      <c r="C4" s="9" t="s">
         <v>137</v>
       </c>
-    </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A4" s="33"/>
-      <c r="B4" s="34"/>
-      <c r="C4" s="9" t="s">
+      <c r="D4" s="9" t="s">
         <v>138</v>
       </c>
-      <c r="D4" s="9" t="s">
+      <c r="E4" s="81"/>
+    </row>
+    <row r="5" spans="1:5" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="A5" s="30"/>
+      <c r="B5" s="32" t="s">
         <v>139</v>
       </c>
-    </row>
-    <row r="5" spans="1:4" ht="43.5" x14ac:dyDescent="0.35">
-      <c r="A5" s="33"/>
-      <c r="B5" s="35" t="s">
+      <c r="C5" s="12" t="s">
         <v>140</v>
       </c>
-      <c r="C5" s="12" t="s">
+      <c r="D5" s="16" t="s">
         <v>141</v>
       </c>
-      <c r="D5" s="16" t="s">
+      <c r="E5" s="81"/>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A6" s="30"/>
+      <c r="B6" s="32"/>
+      <c r="C6" s="9" t="s">
         <v>142</v>
       </c>
-    </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A6" s="33"/>
-      <c r="B6" s="35"/>
-      <c r="C6" s="9" t="s">
+      <c r="D6" s="9" t="s">
         <v>143</v>
       </c>
-      <c r="D6" s="9" t="s">
-        <v>144</v>
-      </c>
+      <c r="E6" s="81"/>
     </row>
   </sheetData>
-  <mergeCells count="3">
+  <mergeCells count="5">
     <mergeCell ref="B3:B4"/>
     <mergeCell ref="B5:B6"/>
     <mergeCell ref="A3:A6"/>
+    <mergeCell ref="B2:C2"/>
+    <mergeCell ref="E3:E6"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="D3" r:id="rId1" xr:uid="{0FEDF6BF-4B1B-49DD-B2E7-AED027AA716D}"/>
@@ -2226,9 +3522,9 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6686655C-2AE1-483D-B494-F33936FFF959}">
-  <dimension ref="A4:D5"/>
+  <dimension ref="A3:E5"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="12" bestFit="1" customWidth="1"/>
@@ -2237,31 +3533,51 @@
     <col min="4" max="4" width="109.7265625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="4" spans="1:4" ht="29" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="B3" s="38" t="s">
+        <v>190</v>
+      </c>
+      <c r="C3" s="37"/>
+      <c r="D3" s="34" t="s">
+        <v>154</v>
+      </c>
+      <c r="E3" s="34" t="s">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" ht="29" x14ac:dyDescent="0.35">
       <c r="A4" s="9" t="s">
+        <v>144</v>
+      </c>
+      <c r="B4" s="9" t="s">
         <v>145</v>
       </c>
-      <c r="B4" s="9" t="s">
+      <c r="C4" s="12" t="s">
         <v>146</v>
       </c>
-      <c r="C4" s="12" t="s">
+      <c r="D4" s="16" t="s">
         <v>147</v>
       </c>
-      <c r="D4" s="16" t="s">
-        <v>148</v>
-      </c>
-    </row>
-    <row r="5" spans="1:4" ht="58" x14ac:dyDescent="0.35">
+      <c r="E4" s="83" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" ht="58" x14ac:dyDescent="0.35">
       <c r="A5" s="9"/>
       <c r="B5" s="9"/>
       <c r="C5" s="12" t="s">
+        <v>148</v>
+      </c>
+      <c r="D5" s="12" t="s">
         <v>149</v>
       </c>
-      <c r="D5" s="12" t="s">
-        <v>150</v>
-      </c>
+      <c r="E5" s="35"/>
     </row>
   </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="B3:C3"/>
+    <mergeCell ref="E4:E5"/>
+  </mergeCells>
   <hyperlinks>
     <hyperlink ref="D4" r:id="rId1" xr:uid="{7F133F5F-A9E3-4A3C-8A06-80CBBF726756}"/>
   </hyperlinks>
@@ -2270,7 +3586,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B577322F-DFF0-420D-9AC6-8B9F87B950F0}">
   <dimension ref="A2:B6"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
@@ -2283,7 +3599,7 @@
         <v>1</v>
       </c>
       <c r="B2" s="19" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
     </row>
     <row r="3" spans="1:2" ht="16" x14ac:dyDescent="0.35">
@@ -2291,7 +3607,7 @@
         <v>2</v>
       </c>
       <c r="B3" s="19" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
     </row>
     <row r="4" spans="1:2" ht="15.5" x14ac:dyDescent="0.35">
@@ -2299,7 +3615,7 @@
         <v>3</v>
       </c>
       <c r="B4" s="19" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
     </row>
     <row r="5" spans="1:2" ht="15.5" x14ac:dyDescent="0.35">
@@ -2307,7 +3623,7 @@
         <v>4</v>
       </c>
       <c r="B5" s="19" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.35">

</xml_diff>